<commit_message>
feat: patch PDF descriptions, fix JSON, add 12 series configs, update report with diagrams and evaluation data, fix schema
</commit_message>
<xml_diff>
--- a/datasets/07_delivery/st_ready/evaluation_report/evaluation_report.xlsx
+++ b/datasets/07_delivery/st_ready/evaluation_report/evaluation_report.xlsx
@@ -39,7 +39,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -64,6 +64,12 @@
         <bgColor rgb="00F44336"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF9800"/>
+        <bgColor rgb="00FF9800"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -83,12 +89,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -486,7 +493,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1</v>
+        <v>296</v>
       </c>
     </row>
     <row r="3">
@@ -496,7 +503,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>1</v>
+        <v>295</v>
       </c>
     </row>
     <row r="4">
@@ -506,7 +513,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>100</v>
+        <v>99.7</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -536,7 +543,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>100</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
@@ -551,7 +558,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>10</v>
+        <v>4733</v>
       </c>
     </row>
     <row r="8">
@@ -561,7 +568,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>10</v>
+        <v>4733</v>
       </c>
     </row>
     <row r="9">
@@ -622,7 +629,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1</v>
+        <v>296</v>
       </c>
     </row>
     <row r="3">
@@ -722,7 +729,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>10</v>
+        <v>4733</v>
       </c>
     </row>
     <row r="10">
@@ -747,7 +754,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>100</v>
+        <v>99.7</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
@@ -798,7 +805,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1</v>
+        <v>296</v>
       </c>
     </row>
     <row r="3">
@@ -823,11 +830,11 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>EXCELLENT</t>
+        <v>81.40000000000001</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>ACCEPTABLE</t>
         </is>
       </c>
     </row>
@@ -838,7 +845,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
@@ -853,7 +860,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>10</v>
+        <v>4733</v>
       </c>
     </row>
     <row r="7">
@@ -863,7 +870,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>60</v>
+        <v>20.9</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
@@ -878,7 +885,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>30</v>
+        <v>24.8</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -893,7 +900,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -903,7 +910,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11">
@@ -913,7 +920,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -923,11 +930,11 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>POOR</t>
+        <v>72.2</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>ACCEPTABLE</t>
         </is>
       </c>
     </row>
@@ -938,7 +945,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -984,7 +991,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1</v>
+        <v>296</v>
       </c>
     </row>
     <row r="3">
@@ -994,7 +1001,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4">
@@ -1004,7 +1011,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
@@ -1019,7 +1026,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1</v>
+        <v>231</v>
       </c>
     </row>
     <row r="6">
@@ -1029,7 +1036,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="7">
@@ -1039,7 +1046,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1085,7 +1092,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1095,7 +1102,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -1105,7 +1112,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -1115,7 +1122,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
@@ -1125,7 +1132,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat : alfred description
</commit_message>
<xml_diff>
--- a/datasets/07_delivery/st_ready/evaluation_report/evaluation_report.xlsx
+++ b/datasets/07_delivery/st_ready/evaluation_report/evaluation_report.xlsx
@@ -39,7 +39,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -54,20 +54,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004CAF50"/>
-        <bgColor rgb="004CAF50"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00F44336"/>
         <bgColor rgb="00F44336"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FF9800"/>
-        <bgColor rgb="00FF9800"/>
+        <fgColor rgb="004CAF50"/>
+        <bgColor rgb="004CAF50"/>
       </patternFill>
     </fill>
   </fills>
@@ -89,13 +83,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -493,7 +486,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>296</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -503,7 +496,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>295</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -513,11 +506,11 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>99.7</v>
+        <v>0</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>EXCELLENT</t>
+          <t>POOR</t>
         </is>
       </c>
     </row>
@@ -528,11 +521,11 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>EXCELLENT</t>
+          <t>POOR</t>
         </is>
       </c>
     </row>
@@ -543,11 +536,11 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>96.59999999999999</v>
+        <v>0</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>EXCELLENT</t>
+          <t>POOR</t>
         </is>
       </c>
     </row>
@@ -558,7 +551,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>4733</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
@@ -568,7 +561,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>4733</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9">
@@ -580,7 +573,7 @@
       <c r="B9" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>EXCELLENT</t>
         </is>
@@ -629,7 +622,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>296</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -639,11 +632,11 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>EXCELLENT</t>
+          <t>POOR</t>
         </is>
       </c>
     </row>
@@ -656,7 +649,7 @@
       <c r="B4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>POOR</t>
         </is>
@@ -671,7 +664,7 @@
       <c r="B5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>POOR</t>
         </is>
@@ -686,7 +679,7 @@
       <c r="B6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>POOR</t>
         </is>
@@ -701,7 +694,7 @@
       <c r="B7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>POOR</t>
         </is>
@@ -716,7 +709,7 @@
       <c r="B8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>POOR</t>
         </is>
@@ -729,7 +722,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>4733</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -741,7 +734,7 @@
       <c r="B10" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>EXCELLENT</t>
         </is>
@@ -754,9 +747,9 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>99.7</v>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+        <v>100</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>EXCELLENT</t>
         </is>
@@ -773,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -805,7 +798,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>296</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -815,11 +808,11 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>EXCELLENT</t>
+          <t>POOR</t>
         </is>
       </c>
     </row>
@@ -830,11 +823,11 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>81.40000000000001</v>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>ACCEPTABLE</t>
+        <v>0</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>POOR</t>
         </is>
       </c>
     </row>
@@ -845,9 +838,9 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>POOR</t>
         </is>
@@ -856,96 +849,56 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Docs Files Total</t>
+          <t>Images Total</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>4733</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Docs Files With Board Pct</t>
+          <t>Images With Desc</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>POOR</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Docs Files With Component Pct</t>
+          <t>Images Failed</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>24.8</v>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>POOR</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Images Total</t>
+          <t>Images Success Pct</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>18</v>
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>POOR</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Images With Desc</t>
+          <t>Images Avg Desc Length</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Images Failed</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Images Success Pct</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>72.2</v>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>ACCEPTABLE</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Images Avg Desc Length</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -959,7 +912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -987,66 +940,13 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Docs Total</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>With Related</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>With Related Pct</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>POOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Without Related</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Avg Related Per Doc</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Max Related</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>3</v>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>NOT_RUN</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1092,7 +992,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1102,7 +1002,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1112,7 +1012,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1122,7 +1022,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1132,7 +1032,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>